<commit_message>
Add 20 blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files: 134
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-drug-discovery.report.xlsx
+++ b/tools/importer/reports/import-drug-discovery.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="125">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,6 +37,51 @@
     <t>url</t>
   </si>
   <si>
+    <t>drug-discovery/about-us.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","tabs-underline","cards-profile","columns-bleed-image","columns-contact"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/about-us</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>section-page</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:31:47.174Z</t>
+  </si>
+  <si>
+    <t>About us - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/about-us.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/get-involved.report.json</t>
+  </si>
+  <si>
+    <t>["toc-on-this-page","toc-on-this-page","columns-title-left","columns-title-left","columns-title-left"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/get-involved</t>
+  </si>
+  <si>
+    <t>text-page</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:31:19.244Z</t>
+  </si>
+  <si>
+    <t>Get involved - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/get-involved.html</t>
+  </si>
+  <si>
     <t>drug-discovery/index.report.json</t>
   </si>
   <si>
@@ -46,19 +91,301 @@
     <t>drug-discovery/index</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
     <t>drug-discovery</t>
   </si>
   <si>
-    <t>2026-10-23T00:44:04.498Z</t>
+    <t>2026-10-23T04:33:28.222Z</t>
   </si>
   <si>
     <t>Centre for Drug Discovery and Innovation - The University of Sydney</t>
   </si>
   <si>
     <t>https://www.sydney.edu.au/drug-discovery/</t>
+  </si>
+  <si>
+    <t>drug-discovery/news-and-events.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","carousel-news","columns-bleed-image","columns-contact"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/news-and-events</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:31:54.104Z</t>
+  </si>
+  <si>
+    <t>News and events - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/news-and-events.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","accordion-plus","cards-cta","columns-bleed-image","columns-title-left","columns-contact"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:32:14.902Z</t>
+  </si>
+  <si>
+    <t>Our research - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/our-research.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/partnerships.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","accordion-plus","carousel-gallery","cards-cta","columns-title-left","columns-contact"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/partnerships</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:33:12.466Z</t>
+  </si>
+  <si>
+    <t>Partnerships - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/partnerships.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/about-us/our-facilities.report.json</t>
+  </si>
+  <si>
+    <t>["toc-on-this-page","toc-on-this-page","columns-title-left","columns-title-left","columns-title-left","columns-title-left"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/about-us/our-facilities</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:31:38.494Z</t>
+  </si>
+  <si>
+    <t>Our facilities - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/about-us/our-facilities.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/get-involved/become-a-member.report.json</t>
+  </si>
+  <si>
+    <t>["toc-on-this-page","embed-formstack"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/get-involved/become-a-member</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:31:24.801Z</t>
+  </si>
+  <si>
+    <t>Become a member - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/get-involved/become-a-member.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/get-involved/researcher-development.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","accordion-plus","carousel-gallery","cards-icon-tile","columns-title-left","columns-contact"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/get-involved/researcher-development</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:33:19.501Z</t>
+  </si>
+  <si>
+    <t>Researcher development - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/get-involved/researcher-development.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/news-and-events/drug-discovery-symposium.report.json</t>
+  </si>
+  <si>
+    <t>["hero-image-overlay","cards-cta","table-key-value","cards-speaker","cards-speaker","cards-speaker"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/news-and-events/drug-discovery-symposium</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:32:08.105Z</t>
+  </si>
+  <si>
+    <t>Drug Discovery Symposium 2025 - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/news-and-events/drug-discovery-symposium.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/news-and-events/news.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","cards-news-list"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/news-and-events/news</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:32:01.369Z</t>
+  </si>
+  <si>
+    <t>News - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/news-and-events/news.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/cancer.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","tabs-underline","tabs-underline","tabs-underline","tabs-underline","columns-contact"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/cancer</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:32:21.856Z</t>
+  </si>
+  <si>
+    <t>Cancer - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/our-research/cancer.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/cardiovascular-disease.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","tabs-underline","tabs-underline","tabs-underline","tabs-underline","tabs-underline","quote-portrait","columns-title-left","columns-contact"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/cardiovascular-disease</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:32:30.285Z</t>
+  </si>
+  <si>
+    <t>Cardiovascular Disease - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/our-research/cardiovascular-disease.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/infectious-diseases.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","tabs-underline","tabs-underline","accordion-plus","quote-portrait","columns-title-left","columns-contact"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/infectious-diseases</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:32:37.494Z</t>
+  </si>
+  <si>
+    <t>Infectious Diseases - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/our-research/infectious-diseases.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/neurological-and-cns-disorders.report.json</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/neurological-and-cns-disorders</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:32:44.521Z</t>
+  </si>
+  <si>
+    <t>Neurological and CNS Disorders - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/our-research/neurological-and-cns-disorders.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/sydney-anti-bacterial-accelerator.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","accordion-plus","columns-title-left","columns-title-left"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/sydney-anti-bacterial-accelerator</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:32:51.471Z</t>
+  </si>
+  <si>
+    <t>Sydney Anti-bacterial Accelerator - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/our-research/sydney-anti-bacterial-accelerator.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/tdp-43-research-cluster.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","accordion-plus","columns-title-left","columns-title-left","columns-title-left"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/tdp-43-research-cluster</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:32:59.301Z</t>
+  </si>
+  <si>
+    <t>TDP-43 Research Cluster - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/our-research/tdp-43-research-cluster.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/what-is-drug-discovery.report.json</t>
+  </si>
+  <si>
+    <t>["hero-orange-split","columns-title-left","columns-title-left","columns-title-left","columns-title-left","columns-title-left","columns-contact"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/our-research/what-is-drug-discovery</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:33:05.717Z</t>
+  </si>
+  <si>
+    <t>What is drug discovery? - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/our-research/what-is-drug-discovery-.html</t>
+  </si>
+  <si>
+    <t>drug-discovery/get-involved/become-a-member/thank-you.report.json</t>
+  </si>
+  <si>
+    <t>["toc-on-this-page"]</t>
+  </si>
+  <si>
+    <t>drug-discovery/get-involved/become-a-member/thank-you</t>
+  </si>
+  <si>
+    <t>2026-10-23T04:31:31.908Z</t>
+  </si>
+  <si>
+    <t>Thank you - The University of Sydney</t>
+  </si>
+  <si>
+    <t>https://www.sydney.edu.au/drug-discovery/get-involved/become-a-member/thank-you.html</t>
   </si>
 </sst>
 </file>
@@ -447,16 +774,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="34" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="1" max="3" width="50" customWidth="1"/>
     <col min="5" max="5" width="16" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
-    <col min="7" max="7" width="50" customWidth="1"/>
-    <col min="8" max="8" width="43" customWidth="1"/>
+    <col min="7" max="8" width="50" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" s="1" customFormat="1" x14ac:dyDescent="0.25">
@@ -509,6 +833,474 @@
       </c>
       <c r="H2" t="s">
         <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
+        <v>17</v>
+      </c>
+      <c r="C3" t="s">
+        <v>18</v>
+      </c>
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>19</v>
+      </c>
+      <c r="F3" t="s">
+        <v>20</v>
+      </c>
+      <c r="G3" t="s">
+        <v>21</v>
+      </c>
+      <c r="H3" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>12</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
+        <v>34</v>
+      </c>
+      <c r="H5" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="s">
+        <v>39</v>
+      </c>
+      <c r="G6" t="s">
+        <v>40</v>
+      </c>
+      <c r="H6" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>42</v>
+      </c>
+      <c r="B7" t="s">
+        <v>43</v>
+      </c>
+      <c r="C7" t="s">
+        <v>44</v>
+      </c>
+      <c r="D7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
+        <v>45</v>
+      </c>
+      <c r="G7" t="s">
+        <v>46</v>
+      </c>
+      <c r="H7" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>49</v>
+      </c>
+      <c r="C8" t="s">
+        <v>50</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" t="s">
+        <v>51</v>
+      </c>
+      <c r="G8" t="s">
+        <v>52</v>
+      </c>
+      <c r="H8" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>55</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>19</v>
+      </c>
+      <c r="F9" t="s">
+        <v>57</v>
+      </c>
+      <c r="G9" t="s">
+        <v>58</v>
+      </c>
+      <c r="H9" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
+        <v>62</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>63</v>
+      </c>
+      <c r="G10" t="s">
+        <v>64</v>
+      </c>
+      <c r="H10" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>66</v>
+      </c>
+      <c r="B11" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" t="s">
+        <v>68</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>12</v>
+      </c>
+      <c r="F11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G11" t="s">
+        <v>70</v>
+      </c>
+      <c r="H11" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>72</v>
+      </c>
+      <c r="B12" t="s">
+        <v>73</v>
+      </c>
+      <c r="C12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>12</v>
+      </c>
+      <c r="F12" t="s">
+        <v>75</v>
+      </c>
+      <c r="G12" t="s">
+        <v>76</v>
+      </c>
+      <c r="H12" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>78</v>
+      </c>
+      <c r="B13" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" t="s">
+        <v>80</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>12</v>
+      </c>
+      <c r="F13" t="s">
+        <v>81</v>
+      </c>
+      <c r="G13" t="s">
+        <v>82</v>
+      </c>
+      <c r="H13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>84</v>
+      </c>
+      <c r="B14" t="s">
+        <v>85</v>
+      </c>
+      <c r="C14" t="s">
+        <v>86</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>12</v>
+      </c>
+      <c r="F14" t="s">
+        <v>87</v>
+      </c>
+      <c r="G14" t="s">
+        <v>88</v>
+      </c>
+      <c r="H14" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>90</v>
+      </c>
+      <c r="B15" t="s">
+        <v>91</v>
+      </c>
+      <c r="C15" t="s">
+        <v>92</v>
+      </c>
+      <c r="D15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E15" t="s">
+        <v>12</v>
+      </c>
+      <c r="F15" t="s">
+        <v>93</v>
+      </c>
+      <c r="G15" t="s">
+        <v>94</v>
+      </c>
+      <c r="H15" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
+        <v>91</v>
+      </c>
+      <c r="C16" t="s">
+        <v>97</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>12</v>
+      </c>
+      <c r="F16" t="s">
+        <v>98</v>
+      </c>
+      <c r="G16" t="s">
+        <v>99</v>
+      </c>
+      <c r="H16" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>101</v>
+      </c>
+      <c r="B17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C17" t="s">
+        <v>103</v>
+      </c>
+      <c r="D17" t="s">
+        <v>11</v>
+      </c>
+      <c r="E17" t="s">
+        <v>12</v>
+      </c>
+      <c r="F17" t="s">
+        <v>104</v>
+      </c>
+      <c r="G17" t="s">
+        <v>105</v>
+      </c>
+      <c r="H17" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B18" t="s">
+        <v>108</v>
+      </c>
+      <c r="C18" t="s">
+        <v>109</v>
+      </c>
+      <c r="D18" t="s">
+        <v>11</v>
+      </c>
+      <c r="E18" t="s">
+        <v>12</v>
+      </c>
+      <c r="F18" t="s">
+        <v>110</v>
+      </c>
+      <c r="G18" t="s">
+        <v>111</v>
+      </c>
+      <c r="H18" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>113</v>
+      </c>
+      <c r="B19" t="s">
+        <v>114</v>
+      </c>
+      <c r="C19" t="s">
+        <v>115</v>
+      </c>
+      <c r="D19" t="s">
+        <v>11</v>
+      </c>
+      <c r="E19" t="s">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>116</v>
+      </c>
+      <c r="G19" t="s">
+        <v>117</v>
+      </c>
+      <c r="H19" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>119</v>
+      </c>
+      <c r="B20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C20" t="s">
+        <v>121</v>
+      </c>
+      <c r="D20" t="s">
+        <v>11</v>
+      </c>
+      <c r="E20" t="s">
+        <v>19</v>
+      </c>
+      <c r="F20" t="s">
+        <v>122</v>
+      </c>
+      <c r="G20" t="s">
+        <v>123</v>
+      </c>
+      <c r="H20" t="s">
+        <v>124</v>
       </c>
     </row>
   </sheetData>

</xml_diff>